<commit_message>
docs: Add master OPNsense SDN guide and update Cursor prompt
</commit_message>
<xml_diff>
--- a/NetOsis_NETWORK_PLAN_UPDATED.xlsx
+++ b/NetOsis_NETWORK_PLAN_UPDATED.xlsx
@@ -746,7 +746,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -811,7 +811,7 @@
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>192.168.10.10</t>
+          <t>192.168.10.31</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
@@ -846,7 +846,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>192.168.10.11</t>
+          <t>192.168.10.32</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
@@ -881,7 +881,7 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>192.168.20.10</t>
+          <t>192.168.20.31</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
@@ -916,7 +916,7 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>192.168.20.11</t>
+          <t>192.168.20.32</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
@@ -951,7 +951,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>192.168.30.10</t>
+          <t>192.168.30.31</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
@@ -986,7 +986,7 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>192.168.30.11</t>
+          <t>192.168.30.32</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
@@ -1072,6 +1072,111 @@
       <c r="G9" s="4" t="inlineStr">
         <is>
           <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>10</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>192.168.10.0/24</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>192.168.10.254</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>192.168.10.10</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>FIN-DECEIVE-01</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Deception (HHP)</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>20</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>192.168.20.0/24</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>192.168.20.254</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>192.168.20.10</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>OPS-DECEIVE-01</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Deception (HHP)</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>30</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>192.168.30.0/24</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>192.168.30.254</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>192.168.30.10</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>ENT-WEB-01 (SSH Honeypot)</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Deception (HHP)</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Active/Tested</t>
         </is>
       </c>
     </row>
@@ -1462,7 +1567,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -1476,182 +1581,246 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Interface/VLAN</t>
+          <t>Interface Identifier</t>
         </is>
       </c>
       <c r="B1" s="3" t="inlineStr">
         <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Type / Device</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
           <t>VLAN ID</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>Subnet</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
-        <is>
-          <t>Gateway</t>
-        </is>
-      </c>
-      <c r="E1" s="3" t="inlineStr">
-        <is>
-          <t>Purpose</t>
-        </is>
-      </c>
       <c r="F1" s="3" t="inlineStr">
         <is>
-          <t>Status</t>
+          <t>Gateway IP</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>FINANCE_VLAN10</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="n">
-        <v>10</v>
+          <t>wan</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>WAN</t>
+        </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>192.168.10.0/24</t>
+          <t>hardware (vtnet1)</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>192.168.10.254</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>172.30.226.0/24</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>Current plan</t>
+          <t>172.30.226.254</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>OPERATIONS_VLAN20</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="n">
-        <v>20</v>
+          <t>lan</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>LAN</t>
+        </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>192.168.20.0/24</t>
+          <t>hardware (vtnet0)</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>192.168.20.254</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>Operations</t>
+          <t>192.168.1.0/24</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>Current plan</t>
+          <t>192.168.1.1</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>ENTERPRISE_VLAN30</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="n">
-        <v>30</v>
+          <t>opt1</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Servers_VLAN250</t>
+        </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>192.168.30.0/24</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>192.168.30.254</t>
-        </is>
+          <t>vlan (vlan0.250)</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>250</v>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Enterprise / public-facing test + deception</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>Current plan</t>
+          <t>TBD</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>SOC_VLAN40</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="n">
-        <v>40</v>
+          <t>opt2</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>FINANCE_VLAN10</t>
+        </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>192.168.40.0/24</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>192.168.40.254</t>
-        </is>
+          <t>vlan (vlan0.10)</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>10</v>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>SOC / telemetry / controller</t>
+          <t>192.168.10.0/24</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>Current plan</t>
+          <t>192.168.10.254</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Existing VLAN 250</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="n">
-        <v>250</v>
+          <t>opt3</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>OPERATIONS_VLAN20</t>
+        </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
+          <t>vlan (vlan0.20)</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>20</v>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Existing VLAN retained</t>
+          <t>192.168.20.0/24</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>Existing</t>
+          <t>192.168.20.254</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>opt4</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ENTERPRISE_VLAN30</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>vlan (vlan0.30)</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>30</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>192.168.30.0/24</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>192.168.30.254</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>opt5</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>SOC_VLAN40</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>vlan (vlan0.40)</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>40</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>192.168.40.0/24</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>192.168.40.254</t>
         </is>
       </c>
     </row>

</xml_diff>